<commit_message>
Publish IG build from TeamCity (62)
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-DIPSBasisPractitionerR4.xlsx
+++ b/docs/StructureDefinition-DIPSBasisPractitionerR4.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4591" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4591" uniqueCount="569">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-15T05:06:55+00:00</t>
+    <t>2026-09-17T19:39:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -989,6 +989,10 @@
   </si>
   <si>
     <t>middlename</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mellomnavn
+</t>
   </si>
   <si>
     <t xml:space="preserve">Extension {http://hl7.no/fhir/StructureDefinition/no-basis-middlename}
@@ -9096,14 +9100,14 @@
         <v>312</v>
       </c>
       <c r="D62" t="s" s="2">
-        <v>75</v>
+        <v>313</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" t="s" s="2">
         <v>76</v>
       </c>
       <c r="G62" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H62" t="s" s="2">
         <v>75</v>
@@ -9115,13 +9119,13 @@
         <v>75</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -9201,10 +9205,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9230,16 +9234,16 @@
         <v>106</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="N63" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="O63" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>75</v>
@@ -9267,10 +9271,10 @@
         <v>180</v>
       </c>
       <c r="Y63" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Z63" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AA63" t="s" s="2">
         <v>75</v>
@@ -9288,7 +9292,7 @@
         <v>75</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>76</v>
@@ -9303,13 +9307,13 @@
         <v>98</v>
       </c>
       <c r="AK63" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="AM63" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="AN63" t="s" s="2">
         <v>75</v>
@@ -9317,10 +9321,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9346,16 +9350,16 @@
         <v>165</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="N64" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="O64" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>75</v>
@@ -9404,7 +9408,7 @@
         <v>75</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>76</v>
@@ -9419,10 +9423,10 @@
         <v>98</v>
       </c>
       <c r="AK64" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="AM64" t="s" s="2">
         <v>75</v>
@@ -9433,14 +9437,14 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E65" s="2"/>
       <c r="F65" t="s" s="2">
@@ -9462,13 +9466,13 @@
         <v>165</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="N65" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O65" s="2"/>
       <c r="P65" t="s" s="2">
@@ -9518,7 +9522,7 @@
         <v>75</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>76</v>
@@ -9533,13 +9537,13 @@
         <v>98</v>
       </c>
       <c r="AK65" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AL65" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AM65" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="AN65" t="s" s="2">
         <v>75</v>
@@ -9547,14 +9551,14 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E66" s="2"/>
       <c r="F66" t="s" s="2">
@@ -9576,13 +9580,13 @@
         <v>165</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="N66" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
@@ -9632,7 +9636,7 @@
         <v>75</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>76</v>
@@ -9647,13 +9651,13 @@
         <v>98</v>
       </c>
       <c r="AK66" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AL66" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="AM66" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AN66" t="s" s="2">
         <v>75</v>
@@ -9661,10 +9665,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9690,10 +9694,10 @@
         <v>165</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
@@ -9744,7 +9748,7 @@
         <v>75</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>76</v>
@@ -9759,13 +9763,13 @@
         <v>98</v>
       </c>
       <c r="AK67" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AM67" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AN67" t="s" s="2">
         <v>75</v>
@@ -9773,10 +9777,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9802,10 +9806,10 @@
         <v>165</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -9856,7 +9860,7 @@
         <v>75</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>76</v>
@@ -9871,10 +9875,10 @@
         <v>98</v>
       </c>
       <c r="AK68" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>75</v>
@@ -9885,10 +9889,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -9914,14 +9918,14 @@
         <v>216</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="P69" t="s" s="2">
         <v>75</v>
@@ -9970,7 +9974,7 @@
         <v>75</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>76</v>
@@ -9985,10 +9989,10 @@
         <v>98</v>
       </c>
       <c r="AK69" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>222</v>
@@ -9999,10 +10003,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -10025,19 +10029,19 @@
         <v>87</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="N70" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="O70" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>75</v>
@@ -10086,7 +10090,7 @@
         <v>75</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>76</v>
@@ -10101,13 +10105,13 @@
         <v>98</v>
       </c>
       <c r="AK70" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="AM70" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AN70" t="s" s="2">
         <v>75</v>
@@ -10115,10 +10119,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10141,19 +10145,19 @@
         <v>87</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="O71" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P71" t="s" s="2">
         <v>75</v>
@@ -10202,7 +10206,7 @@
         <v>75</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>76</v>
@@ -10217,13 +10221,13 @@
         <v>98</v>
       </c>
       <c r="AK71" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="AL71" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="AM71" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="AN71" t="s" s="2">
         <v>75</v>
@@ -10231,10 +10235,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10260,14 +10264,14 @@
         <v>106</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="P72" t="s" s="2">
         <v>75</v>
@@ -10295,10 +10299,10 @@
         <v>180</v>
       </c>
       <c r="Y72" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="Z72" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AA72" t="s" s="2">
         <v>75</v>
@@ -10316,7 +10320,7 @@
         <v>75</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>76</v>
@@ -10331,13 +10335,13 @@
         <v>98</v>
       </c>
       <c r="AK72" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="AL72" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AM72" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AN72" t="s" s="2">
         <v>75</v>
@@ -10345,10 +10349,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10371,17 +10375,17 @@
         <v>87</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="N73" s="2"/>
       <c r="O73" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="P73" t="s" s="2">
         <v>75</v>
@@ -10430,7 +10434,7 @@
         <v>75</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>76</v>
@@ -10445,13 +10449,13 @@
         <v>98</v>
       </c>
       <c r="AK73" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AL73" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AM73" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AN73" t="s" s="2">
         <v>75</v>
@@ -10459,10 +10463,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10485,17 +10489,17 @@
         <v>75</v>
       </c>
       <c r="K74" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="P74" t="s" s="2">
         <v>75</v>
@@ -10544,7 +10548,7 @@
         <v>75</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>76</v>
@@ -10562,10 +10566,10 @@
         <v>75</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AM74" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="AN74" t="s" s="2">
         <v>75</v>
@@ -10573,10 +10577,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -10599,13 +10603,13 @@
         <v>75</v>
       </c>
       <c r="K75" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -10656,7 +10660,7 @@
         <v>75</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>76</v>
@@ -10671,13 +10675,13 @@
         <v>98</v>
       </c>
       <c r="AK75" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AL75" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="AM75" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="AN75" t="s" s="2">
         <v>75</v>
@@ -10685,10 +10689,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10797,10 +10801,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -10911,14 +10915,14 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" t="s" s="2">
@@ -10940,10 +10944,10 @@
         <v>131</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="N78" t="s" s="2">
         <v>151</v>
@@ -10998,7 +11002,7 @@
         <v>75</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>76</v>
@@ -11027,10 +11031,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11056,14 +11060,14 @@
         <v>155</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="P79" t="s" s="2">
         <v>75</v>
@@ -11112,7 +11116,7 @@
         <v>75</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>76</v>
@@ -11130,7 +11134,7 @@
         <v>75</v>
       </c>
       <c r="AL79" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="AM79" t="s" s="2">
         <v>75</v>
@@ -11141,10 +11145,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11170,10 +11174,10 @@
         <v>186</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -11200,13 +11204,13 @@
         <v>75</v>
       </c>
       <c r="X80" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="Y80" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Z80" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AA80" t="s" s="2">
         <v>75</v>
@@ -11224,7 +11228,7 @@
         <v>75</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>86</v>
@@ -11242,10 +11246,10 @@
         <v>75</v>
       </c>
       <c r="AL80" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="AM80" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="AN80" t="s" s="2">
         <v>75</v>
@@ -11253,10 +11257,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11365,10 +11369,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -11479,10 +11483,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11505,19 +11509,19 @@
         <v>87</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="N83" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O83" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P83" t="s" s="2">
         <v>75</v>
@@ -11564,7 +11568,7 @@
         <v>135</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>76</v>
@@ -11579,10 +11583,10 @@
         <v>98</v>
       </c>
       <c r="AK83" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AL83" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="AM83" t="s" s="2">
         <v>75</v>
@@ -11593,10 +11597,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11705,10 +11709,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -11819,10 +11823,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11848,16 +11852,16 @@
         <v>100</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="N86" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="O86" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>75</v>
@@ -11906,7 +11910,7 @@
         <v>75</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>76</v>
@@ -11921,10 +11925,10 @@
         <v>98</v>
       </c>
       <c r="AK86" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AL86" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AM86" t="s" s="2">
         <v>75</v>
@@ -11935,10 +11939,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -11964,13 +11968,13 @@
         <v>165</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N87" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O87" s="2"/>
       <c r="P87" t="s" s="2">
@@ -12020,7 +12024,7 @@
         <v>75</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>76</v>
@@ -12035,10 +12039,10 @@
         <v>98</v>
       </c>
       <c r="AK87" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AL87" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AM87" t="s" s="2">
         <v>75</v>
@@ -12049,10 +12053,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12078,14 +12082,14 @@
         <v>106</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>75</v>
@@ -12134,7 +12138,7 @@
         <v>75</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>76</v>
@@ -12149,10 +12153,10 @@
         <v>98</v>
       </c>
       <c r="AK88" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AL88" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AM88" t="s" s="2">
         <v>75</v>
@@ -12163,10 +12167,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -12192,14 +12196,14 @@
         <v>165</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P89" t="s" s="2">
         <v>75</v>
@@ -12248,7 +12252,7 @@
         <v>75</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>76</v>
@@ -12263,10 +12267,10 @@
         <v>98</v>
       </c>
       <c r="AK89" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AL89" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="AM89" t="s" s="2">
         <v>75</v>
@@ -12277,10 +12281,10 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -12306,16 +12310,16 @@
         <v>293</v>
       </c>
       <c r="L90" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M90" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="N90" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O90" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P90" t="s" s="2">
         <v>75</v>
@@ -12364,7 +12368,7 @@
         <v>75</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>76</v>
@@ -12379,10 +12383,10 @@
         <v>98</v>
       </c>
       <c r="AK90" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AL90" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AM90" t="s" s="2">
         <v>75</v>
@@ -12393,13 +12397,13 @@
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C91" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D91" t="s" s="2">
         <v>75</v>
@@ -12421,19 +12425,19 @@
         <v>87</v>
       </c>
       <c r="K91" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="N91" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O91" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P91" t="s" s="2">
         <v>75</v>
@@ -12462,7 +12466,7 @@
       </c>
       <c r="Y91" s="2"/>
       <c r="Z91" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="AA91" t="s" s="2">
         <v>75</v>
@@ -12480,7 +12484,7 @@
         <v>75</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>76</v>
@@ -12495,10 +12499,10 @@
         <v>98</v>
       </c>
       <c r="AK91" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AL91" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="AM91" t="s" s="2">
         <v>75</v>
@@ -12509,10 +12513,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12621,10 +12625,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12735,10 +12739,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -12764,23 +12768,23 @@
         <v>100</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="N94" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="O94" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>75</v>
       </c>
       <c r="Q94" s="2"/>
       <c r="R94" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="S94" t="s" s="2">
         <v>75</v>
@@ -12822,7 +12826,7 @@
         <v>75</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>76</v>
@@ -12837,10 +12841,10 @@
         <v>98</v>
       </c>
       <c r="AK94" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AL94" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AM94" t="s" s="2">
         <v>75</v>
@@ -12851,10 +12855,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -12880,13 +12884,13 @@
         <v>165</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -12936,7 +12940,7 @@
         <v>75</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>76</v>
@@ -12951,10 +12955,10 @@
         <v>98</v>
       </c>
       <c r="AK95" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AL95" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AM95" t="s" s="2">
         <v>75</v>
@@ -12965,10 +12969,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -12994,14 +12998,14 @@
         <v>106</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>75</v>
@@ -13050,7 +13054,7 @@
         <v>75</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>76</v>
@@ -13065,10 +13069,10 @@
         <v>98</v>
       </c>
       <c r="AK96" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AL96" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AM96" t="s" s="2">
         <v>75</v>
@@ -13079,10 +13083,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13108,14 +13112,14 @@
         <v>165</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>75</v>
@@ -13164,7 +13168,7 @@
         <v>75</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>76</v>
@@ -13179,10 +13183,10 @@
         <v>98</v>
       </c>
       <c r="AK97" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AL97" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="AM97" t="s" s="2">
         <v>75</v>
@@ -13193,10 +13197,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13222,16 +13226,16 @@
         <v>293</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="N98" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O98" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>75</v>
@@ -13280,7 +13284,7 @@
         <v>75</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>76</v>
@@ -13295,10 +13299,10 @@
         <v>98</v>
       </c>
       <c r="AK98" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AL98" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AM98" t="s" s="2">
         <v>75</v>
@@ -13309,13 +13313,13 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C99" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D99" t="s" s="2">
         <v>75</v>
@@ -13337,19 +13341,19 @@
         <v>87</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>75</v>
@@ -13378,7 +13382,7 @@
       </c>
       <c r="Y99" s="2"/>
       <c r="Z99" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="AA99" t="s" s="2">
         <v>75</v>
@@ -13396,7 +13400,7 @@
         <v>75</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>76</v>
@@ -13411,10 +13415,10 @@
         <v>98</v>
       </c>
       <c r="AK99" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AL99" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="AM99" t="s" s="2">
         <v>75</v>
@@ -13425,10 +13429,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13537,10 +13541,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -13651,10 +13655,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -13680,23 +13684,23 @@
         <v>100</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="N102" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="O102" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P102" t="s" s="2">
         <v>75</v>
       </c>
       <c r="Q102" s="2"/>
       <c r="R102" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="S102" t="s" s="2">
         <v>75</v>
@@ -13738,7 +13742,7 @@
         <v>75</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>76</v>
@@ -13753,10 +13757,10 @@
         <v>98</v>
       </c>
       <c r="AK102" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AL102" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AM102" t="s" s="2">
         <v>75</v>
@@ -13767,10 +13771,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -13796,13 +13800,13 @@
         <v>165</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
@@ -13852,7 +13856,7 @@
         <v>75</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>76</v>
@@ -13867,10 +13871,10 @@
         <v>98</v>
       </c>
       <c r="AK103" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AL103" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AM103" t="s" s="2">
         <v>75</v>
@@ -13881,10 +13885,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -13910,14 +13914,14 @@
         <v>106</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="N104" s="2"/>
       <c r="O104" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P104" t="s" s="2">
         <v>75</v>
@@ -13966,7 +13970,7 @@
         <v>75</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>76</v>
@@ -13981,10 +13985,10 @@
         <v>98</v>
       </c>
       <c r="AK104" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AL104" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AM104" t="s" s="2">
         <v>75</v>
@@ -13995,10 +13999,10 @@
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -14024,14 +14028,14 @@
         <v>165</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N105" s="2"/>
       <c r="O105" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P105" t="s" s="2">
         <v>75</v>
@@ -14080,7 +14084,7 @@
         <v>75</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>76</v>
@@ -14095,10 +14099,10 @@
         <v>98</v>
       </c>
       <c r="AK105" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AL105" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="AM105" t="s" s="2">
         <v>75</v>
@@ -14109,10 +14113,10 @@
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -14138,16 +14142,16 @@
         <v>293</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="N106" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O106" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P106" t="s" s="2">
         <v>75</v>
@@ -14196,7 +14200,7 @@
         <v>75</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>76</v>
@@ -14211,10 +14215,10 @@
         <v>98</v>
       </c>
       <c r="AK106" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AL106" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AM106" t="s" s="2">
         <v>75</v>
@@ -14225,13 +14229,13 @@
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C107" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D107" t="s" s="2">
         <v>75</v>
@@ -14253,19 +14257,19 @@
         <v>87</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="N107" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O107" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P107" t="s" s="2">
         <v>75</v>
@@ -14294,7 +14298,7 @@
       </c>
       <c r="Y107" s="2"/>
       <c r="Z107" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="AA107" t="s" s="2">
         <v>75</v>
@@ -14312,7 +14316,7 @@
         <v>75</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>76</v>
@@ -14327,10 +14331,10 @@
         <v>98</v>
       </c>
       <c r="AK107" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AL107" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="AM107" t="s" s="2">
         <v>75</v>
@@ -14341,10 +14345,10 @@
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14453,10 +14457,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14567,10 +14571,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -14596,23 +14600,23 @@
         <v>100</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="N110" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="O110" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P110" t="s" s="2">
         <v>75</v>
       </c>
       <c r="Q110" s="2"/>
       <c r="R110" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="S110" t="s" s="2">
         <v>75</v>
@@ -14654,7 +14658,7 @@
         <v>75</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>76</v>
@@ -14669,10 +14673,10 @@
         <v>98</v>
       </c>
       <c r="AK110" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AL110" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AM110" t="s" s="2">
         <v>75</v>
@@ -14683,10 +14687,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -14712,13 +14716,13 @@
         <v>165</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N111" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O111" s="2"/>
       <c r="P111" t="s" s="2">
@@ -14768,7 +14772,7 @@
         <v>75</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>76</v>
@@ -14783,10 +14787,10 @@
         <v>98</v>
       </c>
       <c r="AK111" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AL111" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AM111" t="s" s="2">
         <v>75</v>
@@ -14797,10 +14801,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -14826,14 +14830,14 @@
         <v>106</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P112" t="s" s="2">
         <v>75</v>
@@ -14882,7 +14886,7 @@
         <v>75</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>76</v>
@@ -14897,10 +14901,10 @@
         <v>98</v>
       </c>
       <c r="AK112" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AM112" t="s" s="2">
         <v>75</v>
@@ -14911,10 +14915,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -14940,14 +14944,14 @@
         <v>165</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P113" t="s" s="2">
         <v>75</v>
@@ -14996,7 +15000,7 @@
         <v>75</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>76</v>
@@ -15011,10 +15015,10 @@
         <v>98</v>
       </c>
       <c r="AK113" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="AM113" t="s" s="2">
         <v>75</v>
@@ -15025,10 +15029,10 @@
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -15054,16 +15058,16 @@
         <v>293</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="N114" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O114" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P114" t="s" s="2">
         <v>75</v>
@@ -15112,7 +15116,7 @@
         <v>75</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>76</v>
@@ -15127,10 +15131,10 @@
         <v>98</v>
       </c>
       <c r="AK114" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AL114" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AM114" t="s" s="2">
         <v>75</v>
@@ -15141,13 +15145,13 @@
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C115" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D115" t="s" s="2">
         <v>75</v>
@@ -15169,19 +15173,19 @@
         <v>87</v>
       </c>
       <c r="K115" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="N115" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="O115" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="P115" t="s" s="2">
         <v>75</v>
@@ -15230,7 +15234,7 @@
         <v>75</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>76</v>
@@ -15245,10 +15249,10 @@
         <v>98</v>
       </c>
       <c r="AK115" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="AM115" t="s" s="2">
         <v>75</v>
@@ -15259,10 +15263,10 @@
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -15371,10 +15375,10 @@
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15485,10 +15489,10 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -15514,23 +15518,23 @@
         <v>100</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="N118" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="O118" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P118" t="s" s="2">
         <v>75</v>
       </c>
       <c r="Q118" s="2"/>
       <c r="R118" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="S118" t="s" s="2">
         <v>75</v>
@@ -15572,7 +15576,7 @@
         <v>75</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>76</v>
@@ -15587,10 +15591,10 @@
         <v>98</v>
       </c>
       <c r="AK118" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AL118" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AM118" t="s" s="2">
         <v>75</v>
@@ -15601,10 +15605,10 @@
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -15630,13 +15634,13 @@
         <v>165</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N119" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O119" s="2"/>
       <c r="P119" t="s" s="2">
@@ -15686,7 +15690,7 @@
         <v>75</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>76</v>
@@ -15701,10 +15705,10 @@
         <v>98</v>
       </c>
       <c r="AK119" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AL119" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AM119" t="s" s="2">
         <v>75</v>
@@ -15715,10 +15719,10 @@
     </row>
     <row r="120">
       <c r="A120" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -15744,14 +15748,14 @@
         <v>106</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M120" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P120" t="s" s="2">
         <v>75</v>
@@ -15800,7 +15804,7 @@
         <v>75</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>76</v>
@@ -15815,10 +15819,10 @@
         <v>98</v>
       </c>
       <c r="AK120" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AL120" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AM120" t="s" s="2">
         <v>75</v>
@@ -15829,10 +15833,10 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -15858,14 +15862,14 @@
         <v>165</v>
       </c>
       <c r="L121" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M121" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P121" t="s" s="2">
         <v>75</v>
@@ -15914,7 +15918,7 @@
         <v>75</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>76</v>
@@ -15929,10 +15933,10 @@
         <v>98</v>
       </c>
       <c r="AK121" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="AL121" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="AM121" t="s" s="2">
         <v>75</v>
@@ -15943,10 +15947,10 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -15972,16 +15976,16 @@
         <v>293</v>
       </c>
       <c r="L122" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M122" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="N122" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O122" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="P122" t="s" s="2">
         <v>75</v>
@@ -16030,7 +16034,7 @@
         <v>75</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>76</v>
@@ -16045,10 +16049,10 @@
         <v>98</v>
       </c>
       <c r="AK122" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AL122" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AM122" t="s" s="2">
         <v>75</v>
@@ -16059,10 +16063,10 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -16088,16 +16092,16 @@
         <v>165</v>
       </c>
       <c r="L123" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="M123" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="N123" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="O123" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="P123" t="s" s="2">
         <v>75</v>
@@ -16146,7 +16150,7 @@
         <v>75</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>76</v>
@@ -16161,10 +16165,10 @@
         <v>98</v>
       </c>
       <c r="AK123" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AL123" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AM123" t="s" s="2">
         <v>75</v>
@@ -16175,10 +16179,10 @@
     </row>
     <row r="124">
       <c r="A124" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -16204,14 +16208,14 @@
         <v>216</v>
       </c>
       <c r="L124" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="M124" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="N124" s="2"/>
       <c r="O124" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="P124" t="s" s="2">
         <v>75</v>
@@ -16260,7 +16264,7 @@
         <v>75</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>76</v>
@@ -16278,10 +16282,10 @@
         <v>75</v>
       </c>
       <c r="AL124" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="AM124" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="AN124" t="s" s="2">
         <v>75</v>
@@ -16289,10 +16293,10 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -16318,10 +16322,10 @@
         <v>224</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="M125" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="N125" s="2"/>
       <c r="O125" s="2"/>
@@ -16372,7 +16376,7 @@
         <v>75</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>76</v>
@@ -16390,7 +16394,7 @@
         <v>75</v>
       </c>
       <c r="AL125" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="AM125" t="s" s="2">
         <v>75</v>
@@ -16401,10 +16405,10 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -16430,16 +16434,16 @@
         <v>186</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="N126" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="O126" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="P126" t="s" s="2">
         <v>75</v>
@@ -16488,7 +16492,7 @@
         <v>75</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>76</v>
@@ -16503,13 +16507,13 @@
         <v>98</v>
       </c>
       <c r="AK126" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="AL126" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="AM126" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="AN126" t="s" s="2">
         <v>75</v>

</xml_diff>